<commit_message>
API updates: guide parity fixes, auth updates, and STAaH certification artifacts
</commit_message>
<xml_diff>
--- a/ChannelConnectAPI_Certification_TestCase V2.xlsx
+++ b/ChannelConnectAPI_Certification_TestCase V2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STAAH\Desktop\TEMPLETS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\dvi_fullstack\api.dvi.travel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C22E6D-3DE6-43D3-887B-A67F58BD98A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC36113-2AB8-453C-887A-C8A69B732F53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ARI Tests" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="82">
   <si>
     <t>STAAH – ChannelConnect API Integration (V2)</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Fetch ARI for Single date</t>
   </si>
   <si>
-    <t>Please share Response in a separate text file</t>
-  </si>
-  <si>
     <t>Booking ID / Reservation Id</t>
   </si>
   <si>
@@ -68,9 +65,6 @@
   </si>
   <si>
     <t>Pre-Book or Check availability before modification</t>
-  </si>
-  <si>
-    <t>Modify</t>
   </si>
   <si>
     <t>Cancel</t>
@@ -151,6 +145,177 @@
       </rPr>
       <t>With an Extra Adult/Child (If Supported Extras)</t>
     </r>
+  </si>
+  <si>
+    <t>2026-04-10 04:51:13 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"property_info","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"checkintime":"02:00 pm","checkouttime":"12:00 am","child_age":"0","contactinfo":{"addressline":"Surat","city":"Adoni","country":"India","email":"uday@staah.com","fax":"","latitude":"21.17024","location":"Surat","longitude":"72.831061","state":"Andhra Pradesh","telephone":"9898989898","zip":"395009"},"currency":"AED","infant_age":"0","propertyname":"Test Property for Channel Connect Partners - Development","trackingId":"8242F0C5-69E8-49CF-8DBC-10167ABEB6D1"}</t>
+  </si>
+  <si>
+    <t>2026-04-10 04:51:14 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"roomrate_info","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"roomtypes" : [{"roomtype":"Double","max_guest":"6","roomsize":"200:SqM","bedding":[{"bed_type":"1 Queen","beds":"1"},{"bed_type":"1 King","beds":"1"}],"total_room":"20","no_of_child":"3","roomname":"Serenity Chamber","room_images":[],"rackrate":"15000","roomtype_view":"Garden view","max_adult":"3","default_inventory":"0","OTA_room_id":"DELUXE","room_id":"166446","dormitory":"","facilities":[{"amenities":["Balcony","Courtyard","Electronic Door Lock"],"amenitytype":"Room Features &amp; Facilities"},{"amenities":["Dryer","Iron &amp; ironing board"],"amenitytype":"Laundry Facilities"},{"amenitytype":"General Amenities","amenities":["Alarm Clock","Bathrobes","Parking"]},{"amenities":["In-room Spa Bath / Jacuzzi"],"amenitytype":"Bathroom Features"},{"amenitytype":"Climate control","amenities":["Air-conditioning"]},{"amenities":["Refrigerator - Bar Size","Tea/Coffee Making facilities"],"amenitytype":"Kitchen Features"},{"amenities":["TV","Netflix"],"amenitytype":"Entertainment"},{"amenities":["FREE WiFi"],"amenitytype":"Internet"}],"description":"Serenity Chamber"}],"rateplans" : [{"validity":[],"smart_price_flag":"","default_maximum_stay":"99","extra_adult_rate":"0","cancelpolicy_id":"","cancellation_policy":"","mealplan":"Room only","OTA_rate_id":"ROOM","ratename":"Continental Plan","nightType":"R","extra_child_rate":"0","rate_id":"3080557","description":"Room Only","applicable_guest":"1","fees":{"Cleaning_fees":"0"},"ignore_tax_flag":"","default_minimum_night":"1"}],"room_rate_mapping" :	[{"rate_id":"3080557","mapping_name":"Continental Plan","OTA_rate_id":"ROOM","room_id":"166446","OTA_room_id":"DELUXE"}], "trackingId" : "02A8E567-C424-4CEC-822C-C874CC0AE7C6"}</t>
+  </si>
+  <si>
+    <t>2026-04-10 04:51:15 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-04-10","to_date":"2026-04-10","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-04-10","inventory":"6","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"77089BC5-EDE4-4D4B-862E-1F2D6C9C90CC"}</t>
+  </si>
+  <si>
+    <t>2026-04-10 04:51:16 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-04-15","to_date":"2026-05-12","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-04-15","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-16","inventory":"5","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-17","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-18","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-19","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-20","inventory":"2","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-21","inventory":"3","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-22","inventory":"2","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-23","inventory":"3","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-24","inventory":"6","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-25","inventory":"6","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-26","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-27","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-28","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-29","inventory":"5","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-04-30","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-01","inventory":"6","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-02","inventory":"6","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-03","inventory":"6","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-04","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-05","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-06","inventory":"5","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-07","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-08","inventory":"6","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-09","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-05-10","inventory":"0","stopsell":"Y"},{"cta":"N","ctd":"N","date":"2026-05-11","inventory":"0","stopsell":"Y"},{"cta":"N","ctd":"N","date":"2026-05-12","inventory":"0","stopsell":"Y"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"B1EA0B83-3733-48FF-8A87-F712BF502E10"}</t>
+  </si>
+  <si>
+    <t>2026-04-10 04:51:17 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-06-01","to_date":"2026-06-10","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-06-01","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-02","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-03","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-04","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-05","inventory":"6","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-06","inventory":"7","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-07","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-08","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-09","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-06-10","inventory":"7","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"3C82F75D-026E-4BC2-8D54-FC93A019AA66"}</t>
+  </si>
+  <si>
+    <t>2026-04-10 04:51:18 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"year_info_ARR","version":"2"}</t>
+  </si>
+  <si>
+    <t>Please refer staah-certification-output/ari-response-samples.txt (TC-06 exact full response).</t>
+  </si>
+  <si>
+    <t>DVI-CERT-S1-1775782282316</t>
+  </si>
+  <si>
+    <t>2026-04-10 00:51:22 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-07-20","to_date":"2026-07-20","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-07-20","inventory":"4","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"F551E0B7-BF57-44C1-8F07-2CA3A593558C"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-07-29T06:00:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S1-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"1240","totaltax":"120","currencycode":"INR","status":"Confirm","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-07-20","departure_date":"2026-07-21","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-07-20","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"120"}],"amountaftertax":"1200","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"2"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>{"status":"ERR","body":"Request timeout after 20000ms"}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-07-21","to_date":"2026-07-21","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-07-21","inventory":"8","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"48559C6D-83AD-4E94-8FC2-02D7C024BA82"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-07-29T06:15:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S1-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"1240","totaltax":"120","currencycode":"INR","status":"Modified","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-07-21","departure_date":"2026-07-22","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-07-21","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"120"}],"amountaftertax":"1200","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"2"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>Modified</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-07-29T06:20:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S1-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"1240","totaltax":"120","currencycode":"INR","status":"Cancel","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-07-21","departure_date":"2026-07-22","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-07-21","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"120"}],"amountaftertax":"1200","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"2"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>DVI-CERT-S2-1775782282316</t>
+  </si>
+  <si>
+    <t>2026-04-10 00:51:40 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-08-10","to_date":"2026-08-10","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-08-10","inventory":"8","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"29AFEA37-7B9C-413B-8674-A0B95C022D6A"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-08-01T07:00:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S2-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"1340","totaltax":"140","currencycode":"INR","status":"Confirm","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-08-10","departure_date":"2026-08-11","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-08-10","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"1","extraAdultRate":"100","extraChildRate":"100"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"140"}],"amountaftertax":"1300","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"3"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-08-11","to_date":"2026-08-11","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-08-11","inventory":"8","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"CBC6308F-CF2C-4659-8ABF-F2AFA480B6F4"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-08-01T07:15:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S2-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"1340","totaltax":"140","currencycode":"INR","status":"Modified","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-08-11","departure_date":"2026-08-12","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-08-11","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"1","extraAdultRate":"100","extraChildRate":"100"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"140"}],"amountaftertax":"1300","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"3"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-08-01T07:20:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S2-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"1340","totaltax":"140","currencycode":"INR","status":"Cancel","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-08-11","departure_date":"2026-08-12","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-08-11","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"1","extraAdultRate":"100","extraChildRate":"100"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"140"}],"amountaftertax":"1300","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"3"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>DVI-CERT-S3-1775782282316</t>
+  </si>
+  <si>
+    <t>2026-04-10 00:51:58 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-09-01","to_date":"2026-09-03","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-09-01","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-09-02","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-09-03","inventory":"8","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"0C95C349-BE73-454E-82CB-7ED038E3166D"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-09-01T08:00:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S3-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"2240","totaltax":"220","currencycode":"INR","status":"Confirm","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-09-01","departure_date":"2026-09-03","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-09-01","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"220"}],"amountaftertax":"2100","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"2"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-09-02","to_date":"2026-09-04","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-09-02","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-09-03","inventory":"8","stopsell":"N"},{"cta":"N","ctd":"N","date":"2026-09-04","inventory":"6","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"E2340689-C177-4AAC-82DC-D3713E79006F"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-09-01T08:15:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S3-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"2360","totaltax":"240","currencycode":"INR","status":"Modified","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-09-02","departure_date":"2026-09-04","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-09-02","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"240"}],"amountaftertax":"2200","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"2"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-09-01T08:20:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S3-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"2360","totaltax":"240","currencycode":"INR","status":"Cancel","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-09-02","departure_date":"2026-09-04","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-09-02","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"240"}],"amountaftertax":"2200","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"2"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>DVI-CERT-S4-1775782282316</t>
+  </si>
+  <si>
+    <t>2026-04-10 00:52:17 GMT</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-10-05","to_date":"2026-10-05","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-10-05","inventory":"10","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"73F94B8A-39E9-45AE-8D78-C248DF7509C0"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-10-01T09:00:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S4-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"2560","totaltax":"260","currencycode":"INR","status":"Confirm","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-10-05","departure_date":"2026-10-06","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-10-05","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"260"}],"amountaftertax":"2400","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"4"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","room_id":"DELUXE","rate_id":"ROOM","action":"ARR_info","from_date":"2026-10-06","to_date":"2026-10-06","version":"2"}</t>
+  </si>
+  <si>
+    <t>{"status":200,"body":{"currency":"AED","data":[{"cta":"N","ctd":"N","date":"2026-10-06","inventory":"11","stopsell":"N"}],"propertyid":"STAAHTESTHOTEL1","rate_id":"ROOM","room_id":"DELUXE","trackingId":"5774B0F3-55BC-4434-846B-072BD190B3BA"}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-10-01T09:15:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S4-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"2680","totaltax":"280","currencycode":"INR","status":"Modified","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-10-06","departure_date":"2026-10-07","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-10-06","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"280"}],"amountaftertax":"2500","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"4"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>{"propertyid":"STAAHTESTHOTEL1","apikey":"Le4-E6F-1F2RB-xZ8a-Oms-jrXIQ-7w73FIH","action":"reservation_info","version":"2","reservations":{"reservation":[{"reservation_datetime":"2026-10-01T09:20:00","propertyname":"STAAH TEST","reservation_id":"DVI-CERT-S4-1775782282316","payment_required":"15","payment_type":"Hotel Collect","commissionamount":"0.00","discountamount":"0.00","deposit":"0.00","totalamountaftertax":"2680","totaltax":"280","currencycode":"INR","status":"Cancel","customer":{"address":"Ring Road","city":"Surat","country":"India","email":"rk@staah.com","salutation":"Mr.","first_name":"Test","last_name":"Test","remarks":"Please Provide Wine Upon Checking and Do not Disturb","telephone":"+91 97734 84053","zip":"395004"},"paymentcarddetail":{"CardHolderName":"Test STAAH","CardType":"MC","ExpireDate":"07/28","CardNumber":"4111111111111111","cvv":"123"},"room":[{"arrival_date":"2026-10-06","departure_date":"2026-10-07","room_id":"DELUXE","room_name":"Studio","price":[{"date":"2026-10-06","rate_id":"ROOM","rate_name":"Test MK","amountaftertax":"1100","extraGuests":{"extraAdult":"1","extraChild":"0","extraAdultRate":"100","extraChildRate":"0"}}],"salutation":"Mr.","first_name":"Test","last_name":"Test","taxes":[{"name":"service charge","value":"280"}],"amountaftertax":"2500","remarks":"No Smoking","GuestCount":[{"AgeQualifyingCode":"10","Count":"4"}]}],"POS":"TEST","extraData":[{"name":"Key","value":"Value of key"}]}]}}</t>
+  </si>
+  <si>
+    <t>Please refer staah-booking-summary-latest.json for full response set.</t>
   </si>
 </sst>
 </file>
@@ -421,6 +586,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -429,24 +612,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -949,16 +1114,16 @@
     <tabColor rgb="FFF79646"/>
   </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="34.54296875" customWidth="1"/>
+    <col min="1" max="1" width="34.5546875" customWidth="1"/>
     <col min="2" max="2" width="48" style="1" customWidth="1"/>
-    <col min="3" max="3" width="42.7265625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="32.54296875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="28.81640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="42.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="32.5546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="28.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="67" customHeight="1">
+    <row r="1" spans="1:5" ht="67.05" customHeight="1">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -969,14 +1134,14 @@
     </row>
     <row r="2" spans="1:5" ht="24" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
       <c r="D2" s="21"/>
       <c r="E2" s="21"/>
     </row>
-    <row r="3" spans="1:5" s="5" customFormat="1" ht="18">
+    <row r="3" spans="1:5" s="5" customFormat="1" ht="17.399999999999999">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -993,72 +1158,106 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="5" customFormat="1" ht="59.15" customHeight="1">
+    <row r="4" spans="1:5" s="5" customFormat="1" ht="59.1" customHeight="1">
       <c r="A4" s="6">
         <v>1</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-    </row>
-    <row r="5" spans="1:5" s="5" customFormat="1" ht="59.15" customHeight="1">
+        <v>16</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="5" customFormat="1" ht="59.1" customHeight="1">
       <c r="A5" s="6">
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-    </row>
-    <row r="6" spans="1:5" s="5" customFormat="1" ht="59.15" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="5" customFormat="1" ht="59.1" customHeight="1">
       <c r="A6" s="6">
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-    </row>
-    <row r="7" spans="1:5" s="5" customFormat="1" ht="59.15" customHeight="1">
+      <c r="C6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="5" customFormat="1" ht="59.1" customHeight="1">
       <c r="A7" s="6">
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-    </row>
-    <row r="8" spans="1:5" s="5" customFormat="1" ht="59.15" customHeight="1">
+        <v>19</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="5" customFormat="1" ht="59.1" customHeight="1">
       <c r="A8" s="6">
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-    </row>
-    <row r="9" spans="1:5" s="5" customFormat="1" ht="59.15" customHeight="1">
+        <v>20</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="5" customFormat="1" ht="59.1" customHeight="1">
       <c r="A9" s="6">
         <v>6</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
+        <v>18</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>41</v>
+      </c>
       <c r="E9" s="10" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="69" customHeight="1">
@@ -1068,7 +1267,7 @@
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
     </row>
-    <row r="11" spans="1:5" ht="14.15" customHeight="1"/>
+    <row r="11" spans="1:5" ht="14.1" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
@@ -1090,14 +1289,14 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="20.54296875" customWidth="1"/>
-    <col min="2" max="2" width="40.7265625" customWidth="1"/>
-    <col min="3" max="3" width="42.7265625" customWidth="1"/>
-    <col min="4" max="4" width="39.81640625" customWidth="1"/>
-    <col min="5" max="5" width="58.08984375" customWidth="1"/>
-    <col min="6" max="7" width="28.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.5546875" customWidth="1"/>
+    <col min="2" max="2" width="40.77734375" customWidth="1"/>
+    <col min="3" max="3" width="42.77734375" customWidth="1"/>
+    <col min="4" max="4" width="39.77734375" customWidth="1"/>
+    <col min="5" max="5" width="58.109375" customWidth="1"/>
+    <col min="6" max="7" width="28.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="66" customHeight="1">
@@ -1113,7 +1312,7 @@
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1">
       <c r="A2" s="31" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
@@ -1131,12 +1330,12 @@
       <c r="F3" s="32"/>
       <c r="G3" s="32"/>
     </row>
-    <row r="4" spans="1:7" ht="18">
+    <row r="4" spans="1:7" ht="17.399999999999999">
       <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="16" t="s">
         <v>3</v>
@@ -1145,7 +1344,7 @@
         <v>2</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>4</v>
@@ -1158,240 +1357,338 @@
       <c r="A5" s="33">
         <v>1</v>
       </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="25"/>
+      <c r="B5" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>44</v>
+      </c>
       <c r="D5" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-    </row>
-    <row r="6" spans="1:7" ht="27.65" customHeight="1">
+      <c r="F5" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="27.6" customHeight="1">
       <c r="A6" s="33"/>
       <c r="B6" s="34"/>
       <c r="C6" s="26"/>
       <c r="D6" s="35"/>
       <c r="E6" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-    </row>
-    <row r="7" spans="1:7" ht="27.65" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="27.6" customHeight="1">
       <c r="A7" s="33"/>
       <c r="B7" s="34"/>
       <c r="C7" s="26"/>
       <c r="D7" s="35"/>
       <c r="E7" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-    </row>
-    <row r="8" spans="1:7" ht="27.65" customHeight="1">
+        <v>12</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="27.6" customHeight="1">
       <c r="A8" s="33"/>
       <c r="B8" s="34"/>
       <c r="C8" s="26"/>
       <c r="D8" s="35"/>
       <c r="E8" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-    </row>
-    <row r="9" spans="1:7" ht="27.65" customHeight="1">
+        <v>52</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="27.6" customHeight="1">
       <c r="A9" s="33"/>
       <c r="B9" s="34"/>
       <c r="C9" s="27"/>
       <c r="D9" s="35"/>
       <c r="E9" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-    </row>
-    <row r="10" spans="1:7" ht="27.65" customHeight="1">
-      <c r="A10" s="28">
+        <v>13</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="27.6" customHeight="1">
+      <c r="A10" s="22">
         <v>2</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="22" t="s">
-        <v>26</v>
+      <c r="B10" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>24</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-    </row>
-    <row r="11" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A11" s="29"/>
+        <v>10</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A11" s="23"/>
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
-      <c r="D11" s="23"/>
+      <c r="D11" s="29"/>
       <c r="E11" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-    </row>
-    <row r="12" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A12" s="29"/>
+        <v>11</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A12" s="23"/>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
-      <c r="D12" s="23"/>
+      <c r="D12" s="29"/>
       <c r="E12" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-    </row>
-    <row r="13" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A13" s="29"/>
+        <v>21</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A13" s="23"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
-      <c r="D13" s="23"/>
+      <c r="D13" s="29"/>
       <c r="E13" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-    </row>
-    <row r="14" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A14" s="30"/>
+        <v>52</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A14" s="24"/>
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
-      <c r="D14" s="24"/>
+      <c r="D14" s="30"/>
       <c r="E14" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-    </row>
-    <row r="15" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A15" s="28">
+        <v>13</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A15" s="22">
         <v>3</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="22" t="s">
-        <v>16</v>
+      <c r="B15" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>14</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-    </row>
-    <row r="16" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A16" s="29"/>
+        <v>10</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A16" s="23"/>
       <c r="B16" s="26"/>
       <c r="C16" s="26"/>
-      <c r="D16" s="23"/>
+      <c r="D16" s="29"/>
       <c r="E16" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-    </row>
-    <row r="17" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A17" s="29"/>
+        <v>11</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A17" s="23"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
-      <c r="D17" s="23"/>
+      <c r="D17" s="29"/>
       <c r="E17" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-    </row>
-    <row r="18" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A18" s="29"/>
+        <v>12</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A18" s="23"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
-      <c r="D18" s="23"/>
+      <c r="D18" s="29"/>
       <c r="E18" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-    </row>
-    <row r="19" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A19" s="30"/>
+        <v>52</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A19" s="24"/>
       <c r="B19" s="27"/>
       <c r="C19" s="27"/>
-      <c r="D19" s="24"/>
+      <c r="D19" s="30"/>
       <c r="E19" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A20" s="22">
+        <v>4</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-    </row>
-    <row r="20" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A20" s="28">
-        <v>4</v>
-      </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="22" t="s">
-        <v>17</v>
-      </c>
       <c r="E20" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-    </row>
-    <row r="21" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A21" s="29"/>
+        <v>10</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A21" s="23"/>
       <c r="B21" s="26"/>
       <c r="C21" s="26"/>
-      <c r="D21" s="23"/>
+      <c r="D21" s="29"/>
       <c r="E21" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-    </row>
-    <row r="22" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A22" s="29"/>
+        <v>11</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A22" s="23"/>
       <c r="B22" s="26"/>
       <c r="C22" s="26"/>
-      <c r="D22" s="23"/>
+      <c r="D22" s="29"/>
       <c r="E22" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-    </row>
-    <row r="23" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A23" s="29"/>
+        <v>12</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A23" s="23"/>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
-      <c r="D23" s="23"/>
+      <c r="D23" s="29"/>
       <c r="E23" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-    </row>
-    <row r="24" spans="1:7" ht="26.9" customHeight="1">
-      <c r="A24" s="30"/>
+        <v>52</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="26.85" customHeight="1">
+      <c r="A24" s="24"/>
       <c r="B24" s="27"/>
       <c r="C24" s="27"/>
-      <c r="D24" s="24"/>
+      <c r="D24" s="30"/>
       <c r="E24" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
+        <v>13</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>81</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C15:C19"/>
+    <mergeCell ref="D15:D19"/>
     <mergeCell ref="A20:A24"/>
     <mergeCell ref="B20:B24"/>
     <mergeCell ref="C20:C24"/>
@@ -1408,8 +1705,6 @@
     <mergeCell ref="C10:C14"/>
     <mergeCell ref="A15:A19"/>
     <mergeCell ref="B15:B19"/>
-    <mergeCell ref="C15:C19"/>
-    <mergeCell ref="D15:D19"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>